<commit_message>
updates on ticket correspondence component
</commit_message>
<xml_diff>
--- a/DEEMPPORTAL.WebUI/wwwroot/files/hr-report.xlsx
+++ b/DEEMPPORTAL.WebUI/wwwroot/files/hr-report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOURCE CODE\PROJECT\DEERP\DEERP.WebUI\wwwroot\files\erp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\DAHBASHI ENGINEERING\EMPLOYEE PORTAL\DEEMPPORTAL.WebUI\wwwroot\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD36C6C-87EF-41E2-9567-CDA159FE6DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9F2523-1C27-47A4-B41C-1B83DEB718EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Sno</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>Emergency Contact Name</t>
+  </si>
+  <si>
+    <t>Personal Email</t>
+  </si>
+  <si>
+    <t>Work Email</t>
   </si>
 </sst>
 </file>
@@ -410,7 +416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K169"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.7109375" customWidth="1"/>
@@ -421,10 +427,10 @@
     <col min="8" max="8" width="32.28515625" customWidth="1"/>
     <col min="9" max="9" width="29" customWidth="1"/>
     <col min="10" max="10" width="29.140625" customWidth="1"/>
-    <col min="11" max="11" width="28.42578125" customWidth="1"/>
+    <col min="11" max="13" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -458,8 +464,14 @@
       <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -471,8 +483,10 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -484,8 +498,10 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -497,8 +513,10 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -510,8 +528,10 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -523,8 +543,10 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -536,8 +558,10 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -549,8 +573,10 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -562,8 +588,10 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -575,8 +603,10 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -588,8 +618,10 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -601,8 +633,10 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -614,8 +648,10 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -627,8 +663,10 @@
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -640,8 +678,10 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -653,8 +693,10 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -666,8 +708,10 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -679,8 +723,10 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -692,8 +738,10 @@
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -705,8 +753,10 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -718,8 +768,10 @@
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -731,8 +783,10 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -744,8 +798,10 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -757,8 +813,10 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -770,8 +828,10 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -783,8 +843,10 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -796,8 +858,10 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -809,8 +873,10 @@
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -822,8 +888,10 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -835,8 +903,10 @@
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -848,8 +918,10 @@
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -861,8 +933,10 @@
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -874,8 +948,10 @@
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -887,8 +963,10 @@
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -900,8 +978,10 @@
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -913,8 +993,10 @@
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -926,8 +1008,10 @@
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -939,8 +1023,10 @@
       <c r="I38" s="1"/>
       <c r="J38" s="1"/>
       <c r="K38" s="1"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -952,8 +1038,10 @@
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -965,8 +1053,10 @@
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -978,8 +1068,10 @@
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -991,8 +1083,10 @@
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1004,8 +1098,10 @@
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1017,8 +1113,10 @@
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1030,8 +1128,10 @@
       <c r="I45" s="1"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1043,8 +1143,10 @@
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1056,8 +1158,10 @@
       <c r="I47" s="1"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1069,8 +1173,10 @@
       <c r="I48" s="1"/>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1082,8 +1188,10 @@
       <c r="I49" s="1"/>
       <c r="J49" s="1"/>
       <c r="K49" s="1"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1095,8 +1203,10 @@
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1108,8 +1218,10 @@
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1121,8 +1233,10 @@
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1134,8 +1248,10 @@
       <c r="I53" s="1"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1147,8 +1263,10 @@
       <c r="I54" s="1"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1160,8 +1278,10 @@
       <c r="I55" s="1"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1173,8 +1293,10 @@
       <c r="I56" s="1"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1186,8 +1308,10 @@
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1199,8 +1323,10 @@
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -1212,8 +1338,10 @@
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -1225,8 +1353,10 @@
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -1238,8 +1368,10 @@
       <c r="I61" s="1"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L61" s="1"/>
+      <c r="M61" s="1"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -1251,8 +1383,10 @@
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L62" s="1"/>
+      <c r="M62" s="1"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -1264,8 +1398,10 @@
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L63" s="1"/>
+      <c r="M63" s="1"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -1277,8 +1413,10 @@
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L64" s="1"/>
+      <c r="M64" s="1"/>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -1290,8 +1428,10 @@
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L65" s="1"/>
+      <c r="M65" s="1"/>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>
@@ -1303,8 +1443,10 @@
       <c r="I66" s="1"/>
       <c r="J66" s="1"/>
       <c r="K66" s="1"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L66" s="1"/>
+      <c r="M66" s="1"/>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
       <c r="C67" s="1"/>
@@ -1316,8 +1458,10 @@
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L67" s="1"/>
+      <c r="M67" s="1"/>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -1329,8 +1473,10 @@
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L68" s="1"/>
+      <c r="M68" s="1"/>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
@@ -1342,8 +1488,10 @@
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L69" s="1"/>
+      <c r="M69" s="1"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
@@ -1355,8 +1503,10 @@
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L70" s="1"/>
+      <c r="M70" s="1"/>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
       <c r="C71" s="1"/>
@@ -1368,8 +1518,10 @@
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
       <c r="C72" s="1"/>
@@ -1381,8 +1533,10 @@
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
       <c r="C73" s="1"/>
@@ -1394,8 +1548,10 @@
       <c r="I73" s="1"/>
       <c r="J73" s="1"/>
       <c r="K73" s="1"/>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
@@ -1407,8 +1563,10 @@
       <c r="I74" s="1"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L74" s="1"/>
+      <c r="M74" s="1"/>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
@@ -1420,8 +1578,10 @@
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L75" s="1"/>
+      <c r="M75" s="1"/>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
@@ -1433,8 +1593,10 @@
       <c r="I76" s="1"/>
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L76" s="1"/>
+      <c r="M76" s="1"/>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
@@ -1446,8 +1608,10 @@
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L77" s="1"/>
+      <c r="M77" s="1"/>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
@@ -1459,8 +1623,10 @@
       <c r="I78" s="1"/>
       <c r="J78" s="1"/>
       <c r="K78" s="1"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L78" s="1"/>
+      <c r="M78" s="1"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
@@ -1472,8 +1638,10 @@
       <c r="I79" s="1"/>
       <c r="J79" s="1"/>
       <c r="K79" s="1"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L79" s="1"/>
+      <c r="M79" s="1"/>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
@@ -1485,8 +1653,10 @@
       <c r="I80" s="1"/>
       <c r="J80" s="1"/>
       <c r="K80" s="1"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L80" s="1"/>
+      <c r="M80" s="1"/>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
@@ -1498,8 +1668,10 @@
       <c r="I81" s="1"/>
       <c r="J81" s="1"/>
       <c r="K81" s="1"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L81" s="1"/>
+      <c r="M81" s="1"/>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1"/>
@@ -1511,8 +1683,10 @@
       <c r="I82" s="1"/>
       <c r="J82" s="1"/>
       <c r="K82" s="1"/>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L82" s="1"/>
+      <c r="M82" s="1"/>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
       <c r="C83" s="1"/>
@@ -1524,8 +1698,10 @@
       <c r="I83" s="1"/>
       <c r="J83" s="1"/>
       <c r="K83" s="1"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L83" s="1"/>
+      <c r="M83" s="1"/>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
       <c r="C84" s="1"/>
@@ -1537,8 +1713,10 @@
       <c r="I84" s="1"/>
       <c r="J84" s="1"/>
       <c r="K84" s="1"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L84" s="1"/>
+      <c r="M84" s="1"/>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
       <c r="C85" s="1"/>
@@ -1550,8 +1728,10 @@
       <c r="I85" s="1"/>
       <c r="J85" s="1"/>
       <c r="K85" s="1"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L85" s="1"/>
+      <c r="M85" s="1"/>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
       <c r="C86" s="1"/>
@@ -1563,8 +1743,10 @@
       <c r="I86" s="1"/>
       <c r="J86" s="1"/>
       <c r="K86" s="1"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L86" s="1"/>
+      <c r="M86" s="1"/>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
       <c r="C87" s="1"/>
@@ -1576,8 +1758,10 @@
       <c r="I87" s="1"/>
       <c r="J87" s="1"/>
       <c r="K87" s="1"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L87" s="1"/>
+      <c r="M87" s="1"/>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
       <c r="C88" s="1"/>
@@ -1589,8 +1773,10 @@
       <c r="I88" s="1"/>
       <c r="J88" s="1"/>
       <c r="K88" s="1"/>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L88" s="1"/>
+      <c r="M88" s="1"/>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -1602,8 +1788,10 @@
       <c r="I89" s="1"/>
       <c r="J89" s="1"/>
       <c r="K89" s="1"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L89" s="1"/>
+      <c r="M89" s="1"/>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
       <c r="C90" s="1"/>
@@ -1615,8 +1803,10 @@
       <c r="I90" s="1"/>
       <c r="J90" s="1"/>
       <c r="K90" s="1"/>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L90" s="1"/>
+      <c r="M90" s="1"/>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
       <c r="C91" s="1"/>
@@ -1628,8 +1818,10 @@
       <c r="I91" s="1"/>
       <c r="J91" s="1"/>
       <c r="K91" s="1"/>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L91" s="1"/>
+      <c r="M91" s="1"/>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -1641,8 +1833,10 @@
       <c r="I92" s="1"/>
       <c r="J92" s="1"/>
       <c r="K92" s="1"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
+    </row>
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
       <c r="C93" s="1"/>
@@ -1654,8 +1848,10 @@
       <c r="I93" s="1"/>
       <c r="J93" s="1"/>
       <c r="K93" s="1"/>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
@@ -1667,8 +1863,10 @@
       <c r="I94" s="1"/>
       <c r="J94" s="1"/>
       <c r="K94" s="1"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
@@ -1680,8 +1878,10 @@
       <c r="I95" s="1"/>
       <c r="J95" s="1"/>
       <c r="K95" s="1"/>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L95" s="1"/>
+      <c r="M95" s="1"/>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
@@ -1693,8 +1893,10 @@
       <c r="I96" s="1"/>
       <c r="J96" s="1"/>
       <c r="K96" s="1"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L96" s="1"/>
+      <c r="M96" s="1"/>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
@@ -1706,8 +1908,10 @@
       <c r="I97" s="1"/>
       <c r="J97" s="1"/>
       <c r="K97" s="1"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L97" s="1"/>
+      <c r="M97" s="1"/>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -1719,8 +1923,10 @@
       <c r="I98" s="1"/>
       <c r="J98" s="1"/>
       <c r="K98" s="1"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L98" s="1"/>
+      <c r="M98" s="1"/>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
@@ -1732,8 +1938,10 @@
       <c r="I99" s="1"/>
       <c r="J99" s="1"/>
       <c r="K99" s="1"/>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L99" s="1"/>
+      <c r="M99" s="1"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
       <c r="C100" s="1"/>
@@ -1745,8 +1953,10 @@
       <c r="I100" s="1"/>
       <c r="J100" s="1"/>
       <c r="K100" s="1"/>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L100" s="1"/>
+      <c r="M100" s="1"/>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
       <c r="C101" s="1"/>
@@ -1758,8 +1968,10 @@
       <c r="I101" s="1"/>
       <c r="J101" s="1"/>
       <c r="K101" s="1"/>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L101" s="1"/>
+      <c r="M101" s="1"/>
+    </row>
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -1771,8 +1983,10 @@
       <c r="I102" s="1"/>
       <c r="J102" s="1"/>
       <c r="K102" s="1"/>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L102" s="1"/>
+      <c r="M102" s="1"/>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -1784,8 +1998,10 @@
       <c r="I103" s="1"/>
       <c r="J103" s="1"/>
       <c r="K103" s="1"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L103" s="1"/>
+      <c r="M103" s="1"/>
+    </row>
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -1797,8 +2013,10 @@
       <c r="I104" s="1"/>
       <c r="J104" s="1"/>
       <c r="K104" s="1"/>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L104" s="1"/>
+      <c r="M104" s="1"/>
+    </row>
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
       <c r="C105" s="1"/>
@@ -1810,8 +2028,10 @@
       <c r="I105" s="1"/>
       <c r="J105" s="1"/>
       <c r="K105" s="1"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L105" s="1"/>
+      <c r="M105" s="1"/>
+    </row>
+    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
       <c r="C106" s="1"/>
@@ -1823,8 +2043,10 @@
       <c r="I106" s="1"/>
       <c r="J106" s="1"/>
       <c r="K106" s="1"/>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L106" s="1"/>
+      <c r="M106" s="1"/>
+    </row>
+    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
@@ -1836,8 +2058,10 @@
       <c r="I107" s="1"/>
       <c r="J107" s="1"/>
       <c r="K107" s="1"/>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L107" s="1"/>
+      <c r="M107" s="1"/>
+    </row>
+    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
@@ -1849,8 +2073,10 @@
       <c r="I108" s="1"/>
       <c r="J108" s="1"/>
       <c r="K108" s="1"/>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L108" s="1"/>
+      <c r="M108" s="1"/>
+    </row>
+    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
@@ -1862,8 +2088,10 @@
       <c r="I109" s="1"/>
       <c r="J109" s="1"/>
       <c r="K109" s="1"/>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L109" s="1"/>
+      <c r="M109" s="1"/>
+    </row>
+    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
@@ -1875,8 +2103,10 @@
       <c r="I110" s="1"/>
       <c r="J110" s="1"/>
       <c r="K110" s="1"/>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L110" s="1"/>
+      <c r="M110" s="1"/>
+    </row>
+    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
       <c r="C111" s="1"/>
@@ -1888,8 +2118,10 @@
       <c r="I111" s="1"/>
       <c r="J111" s="1"/>
       <c r="K111" s="1"/>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L111" s="1"/>
+      <c r="M111" s="1"/>
+    </row>
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
       <c r="C112" s="1"/>
@@ -1901,8 +2133,10 @@
       <c r="I112" s="1"/>
       <c r="J112" s="1"/>
       <c r="K112" s="1"/>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L112" s="1"/>
+      <c r="M112" s="1"/>
+    </row>
+    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
@@ -1914,8 +2148,10 @@
       <c r="I113" s="1"/>
       <c r="J113" s="1"/>
       <c r="K113" s="1"/>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L113" s="1"/>
+      <c r="M113" s="1"/>
+    </row>
+    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
@@ -1927,8 +2163,10 @@
       <c r="I114" s="1"/>
       <c r="J114" s="1"/>
       <c r="K114" s="1"/>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L114" s="1"/>
+      <c r="M114" s="1"/>
+    </row>
+    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
@@ -1940,8 +2178,10 @@
       <c r="I115" s="1"/>
       <c r="J115" s="1"/>
       <c r="K115" s="1"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L115" s="1"/>
+      <c r="M115" s="1"/>
+    </row>
+    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
@@ -1953,8 +2193,10 @@
       <c r="I116" s="1"/>
       <c r="J116" s="1"/>
       <c r="K116" s="1"/>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L116" s="1"/>
+      <c r="M116" s="1"/>
+    </row>
+    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
@@ -1966,8 +2208,10 @@
       <c r="I117" s="1"/>
       <c r="J117" s="1"/>
       <c r="K117" s="1"/>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L117" s="1"/>
+      <c r="M117" s="1"/>
+    </row>
+    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
@@ -1979,8 +2223,10 @@
       <c r="I118" s="1"/>
       <c r="J118" s="1"/>
       <c r="K118" s="1"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L118" s="1"/>
+      <c r="M118" s="1"/>
+    </row>
+    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
       <c r="C119" s="1"/>
@@ -1992,8 +2238,10 @@
       <c r="I119" s="1"/>
       <c r="J119" s="1"/>
       <c r="K119" s="1"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L119" s="1"/>
+      <c r="M119" s="1"/>
+    </row>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
       <c r="C120" s="1"/>
@@ -2005,8 +2253,10 @@
       <c r="I120" s="1"/>
       <c r="J120" s="1"/>
       <c r="K120" s="1"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L120" s="1"/>
+      <c r="M120" s="1"/>
+    </row>
+    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
       <c r="C121" s="1"/>
@@ -2018,8 +2268,10 @@
       <c r="I121" s="1"/>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L121" s="1"/>
+      <c r="M121" s="1"/>
+    </row>
+    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
       <c r="C122" s="1"/>
@@ -2031,8 +2283,10 @@
       <c r="I122" s="1"/>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L122" s="1"/>
+      <c r="M122" s="1"/>
+    </row>
+    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
       <c r="C123" s="1"/>
@@ -2044,8 +2298,10 @@
       <c r="I123" s="1"/>
       <c r="J123" s="1"/>
       <c r="K123" s="1"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L123" s="1"/>
+      <c r="M123" s="1"/>
+    </row>
+    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
@@ -2057,8 +2313,10 @@
       <c r="I124" s="1"/>
       <c r="J124" s="1"/>
       <c r="K124" s="1"/>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L124" s="1"/>
+      <c r="M124" s="1"/>
+    </row>
+    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
@@ -2070,8 +2328,10 @@
       <c r="I125" s="1"/>
       <c r="J125" s="1"/>
       <c r="K125" s="1"/>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L125" s="1"/>
+      <c r="M125" s="1"/>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
@@ -2083,8 +2343,10 @@
       <c r="I126" s="1"/>
       <c r="J126" s="1"/>
       <c r="K126" s="1"/>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L126" s="1"/>
+      <c r="M126" s="1"/>
+    </row>
+    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
       <c r="C127" s="1"/>
@@ -2096,8 +2358,10 @@
       <c r="I127" s="1"/>
       <c r="J127" s="1"/>
       <c r="K127" s="1"/>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L127" s="1"/>
+      <c r="M127" s="1"/>
+    </row>
+    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
       <c r="C128" s="1"/>
@@ -2109,8 +2373,10 @@
       <c r="I128" s="1"/>
       <c r="J128" s="1"/>
       <c r="K128" s="1"/>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L128" s="1"/>
+      <c r="M128" s="1"/>
+    </row>
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
       <c r="C129" s="1"/>
@@ -2122,8 +2388,10 @@
       <c r="I129" s="1"/>
       <c r="J129" s="1"/>
       <c r="K129" s="1"/>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L129" s="1"/>
+      <c r="M129" s="1"/>
+    </row>
+    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
       <c r="C130" s="1"/>
@@ -2135,8 +2403,10 @@
       <c r="I130" s="1"/>
       <c r="J130" s="1"/>
       <c r="K130" s="1"/>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L130" s="1"/>
+      <c r="M130" s="1"/>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
       <c r="C131" s="1"/>
@@ -2148,8 +2418,10 @@
       <c r="I131" s="1"/>
       <c r="J131" s="1"/>
       <c r="K131" s="1"/>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L131" s="1"/>
+      <c r="M131" s="1"/>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
       <c r="C132" s="1"/>
@@ -2161,8 +2433,10 @@
       <c r="I132" s="1"/>
       <c r="J132" s="1"/>
       <c r="K132" s="1"/>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L132" s="1"/>
+      <c r="M132" s="1"/>
+    </row>
+    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
       <c r="C133" s="1"/>
@@ -2174,8 +2448,10 @@
       <c r="I133" s="1"/>
       <c r="J133" s="1"/>
       <c r="K133" s="1"/>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L133" s="1"/>
+      <c r="M133" s="1"/>
+    </row>
+    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
@@ -2187,8 +2463,10 @@
       <c r="I134" s="1"/>
       <c r="J134" s="1"/>
       <c r="K134" s="1"/>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L134" s="1"/>
+      <c r="M134" s="1"/>
+    </row>
+    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
@@ -2200,8 +2478,10 @@
       <c r="I135" s="1"/>
       <c r="J135" s="1"/>
       <c r="K135" s="1"/>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L135" s="1"/>
+      <c r="M135" s="1"/>
+    </row>
+    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
@@ -2213,8 +2493,10 @@
       <c r="I136" s="1"/>
       <c r="J136" s="1"/>
       <c r="K136" s="1"/>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L136" s="1"/>
+      <c r="M136" s="1"/>
+    </row>
+    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
       <c r="C137" s="1"/>
@@ -2226,8 +2508,10 @@
       <c r="I137" s="1"/>
       <c r="J137" s="1"/>
       <c r="K137" s="1"/>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L137" s="1"/>
+      <c r="M137" s="1"/>
+    </row>
+    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
       <c r="C138" s="1"/>
@@ -2239,8 +2523,10 @@
       <c r="I138" s="1"/>
       <c r="J138" s="1"/>
       <c r="K138" s="1"/>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L138" s="1"/>
+      <c r="M138" s="1"/>
+    </row>
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -2252,8 +2538,10 @@
       <c r="I139" s="1"/>
       <c r="J139" s="1"/>
       <c r="K139" s="1"/>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L139" s="1"/>
+      <c r="M139" s="1"/>
+    </row>
+    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
       <c r="C140" s="1"/>
@@ -2265,8 +2553,10 @@
       <c r="I140" s="1"/>
       <c r="J140" s="1"/>
       <c r="K140" s="1"/>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L140" s="1"/>
+      <c r="M140" s="1"/>
+    </row>
+    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
       <c r="C141" s="1"/>
@@ -2278,8 +2568,10 @@
       <c r="I141" s="1"/>
       <c r="J141" s="1"/>
       <c r="K141" s="1"/>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L141" s="1"/>
+      <c r="M141" s="1"/>
+    </row>
+    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
       <c r="C142" s="1"/>
@@ -2291,8 +2583,10 @@
       <c r="I142" s="1"/>
       <c r="J142" s="1"/>
       <c r="K142" s="1"/>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L142" s="1"/>
+      <c r="M142" s="1"/>
+    </row>
+    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
       <c r="C143" s="1"/>
@@ -2304,8 +2598,10 @@
       <c r="I143" s="1"/>
       <c r="J143" s="1"/>
       <c r="K143" s="1"/>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L143" s="1"/>
+      <c r="M143" s="1"/>
+    </row>
+    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
       <c r="C144" s="1"/>
@@ -2317,8 +2613,10 @@
       <c r="I144" s="1"/>
       <c r="J144" s="1"/>
       <c r="K144" s="1"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L144" s="1"/>
+      <c r="M144" s="1"/>
+    </row>
+    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
       <c r="C145" s="1"/>
@@ -2330,8 +2628,10 @@
       <c r="I145" s="1"/>
       <c r="J145" s="1"/>
       <c r="K145" s="1"/>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L145" s="1"/>
+      <c r="M145" s="1"/>
+    </row>
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
       <c r="C146" s="1"/>
@@ -2343,8 +2643,10 @@
       <c r="I146" s="1"/>
       <c r="J146" s="1"/>
       <c r="K146" s="1"/>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L146" s="1"/>
+      <c r="M146" s="1"/>
+    </row>
+    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
       <c r="C147" s="1"/>
@@ -2356,8 +2658,10 @@
       <c r="I147" s="1"/>
       <c r="J147" s="1"/>
       <c r="K147" s="1"/>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L147" s="1"/>
+      <c r="M147" s="1"/>
+    </row>
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
       <c r="C148" s="1"/>
@@ -2369,8 +2673,10 @@
       <c r="I148" s="1"/>
       <c r="J148" s="1"/>
       <c r="K148" s="1"/>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L148" s="1"/>
+      <c r="M148" s="1"/>
+    </row>
+    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
       <c r="C149" s="1"/>
@@ -2382,8 +2688,10 @@
       <c r="I149" s="1"/>
       <c r="J149" s="1"/>
       <c r="K149" s="1"/>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L149" s="1"/>
+      <c r="M149" s="1"/>
+    </row>
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
       <c r="C150" s="1"/>
@@ -2395,8 +2703,10 @@
       <c r="I150" s="1"/>
       <c r="J150" s="1"/>
       <c r="K150" s="1"/>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L150" s="1"/>
+      <c r="M150" s="1"/>
+    </row>
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
       <c r="C151" s="1"/>
@@ -2408,8 +2718,10 @@
       <c r="I151" s="1"/>
       <c r="J151" s="1"/>
       <c r="K151" s="1"/>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L151" s="1"/>
+      <c r="M151" s="1"/>
+    </row>
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
       <c r="C152" s="1"/>
@@ -2421,8 +2733,10 @@
       <c r="I152" s="1"/>
       <c r="J152" s="1"/>
       <c r="K152" s="1"/>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L152" s="1"/>
+      <c r="M152" s="1"/>
+    </row>
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
       <c r="C153" s="1"/>
@@ -2434,8 +2748,10 @@
       <c r="I153" s="1"/>
       <c r="J153" s="1"/>
       <c r="K153" s="1"/>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L153" s="1"/>
+      <c r="M153" s="1"/>
+    </row>
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
       <c r="C154" s="1"/>
@@ -2447,8 +2763,10 @@
       <c r="I154" s="1"/>
       <c r="J154" s="1"/>
       <c r="K154" s="1"/>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L154" s="1"/>
+      <c r="M154" s="1"/>
+    </row>
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
       <c r="C155" s="1"/>
@@ -2460,8 +2778,10 @@
       <c r="I155" s="1"/>
       <c r="J155" s="1"/>
       <c r="K155" s="1"/>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L155" s="1"/>
+      <c r="M155" s="1"/>
+    </row>
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -2473,8 +2793,10 @@
       <c r="I156" s="1"/>
       <c r="J156" s="1"/>
       <c r="K156" s="1"/>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L156" s="1"/>
+      <c r="M156" s="1"/>
+    </row>
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
       <c r="C157" s="1"/>
@@ -2486,8 +2808,10 @@
       <c r="I157" s="1"/>
       <c r="J157" s="1"/>
       <c r="K157" s="1"/>
-    </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L157" s="1"/>
+      <c r="M157" s="1"/>
+    </row>
+    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
       <c r="C158" s="1"/>
@@ -2499,8 +2823,10 @@
       <c r="I158" s="1"/>
       <c r="J158" s="1"/>
       <c r="K158" s="1"/>
-    </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L158" s="1"/>
+      <c r="M158" s="1"/>
+    </row>
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
       <c r="C159" s="1"/>
@@ -2512,8 +2838,10 @@
       <c r="I159" s="1"/>
       <c r="J159" s="1"/>
       <c r="K159" s="1"/>
-    </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L159" s="1"/>
+      <c r="M159" s="1"/>
+    </row>
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
       <c r="C160" s="1"/>
@@ -2525,8 +2853,10 @@
       <c r="I160" s="1"/>
       <c r="J160" s="1"/>
       <c r="K160" s="1"/>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L160" s="1"/>
+      <c r="M160" s="1"/>
+    </row>
+    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
       <c r="C161" s="1"/>
@@ -2538,8 +2868,10 @@
       <c r="I161" s="1"/>
       <c r="J161" s="1"/>
       <c r="K161" s="1"/>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L161" s="1"/>
+      <c r="M161" s="1"/>
+    </row>
+    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
       <c r="C162" s="1"/>
@@ -2551,8 +2883,10 @@
       <c r="I162" s="1"/>
       <c r="J162" s="1"/>
       <c r="K162" s="1"/>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L162" s="1"/>
+      <c r="M162" s="1"/>
+    </row>
+    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
@@ -2564,8 +2898,10 @@
       <c r="I163" s="1"/>
       <c r="J163" s="1"/>
       <c r="K163" s="1"/>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L163" s="1"/>
+      <c r="M163" s="1"/>
+    </row>
+    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
@@ -2577,8 +2913,10 @@
       <c r="I164" s="1"/>
       <c r="J164" s="1"/>
       <c r="K164" s="1"/>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L164" s="1"/>
+      <c r="M164" s="1"/>
+    </row>
+    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
@@ -2590,8 +2928,10 @@
       <c r="I165" s="1"/>
       <c r="J165" s="1"/>
       <c r="K165" s="1"/>
-    </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L165" s="1"/>
+      <c r="M165" s="1"/>
+    </row>
+    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -2603,8 +2943,10 @@
       <c r="I166" s="1"/>
       <c r="J166" s="1"/>
       <c r="K166" s="1"/>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L166" s="1"/>
+      <c r="M166" s="1"/>
+    </row>
+    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
       <c r="C167" s="1"/>
@@ -2616,8 +2958,10 @@
       <c r="I167" s="1"/>
       <c r="J167" s="1"/>
       <c r="K167" s="1"/>
-    </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L167" s="1"/>
+      <c r="M167" s="1"/>
+    </row>
+    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
       <c r="C168" s="1"/>
@@ -2629,8 +2973,10 @@
       <c r="I168" s="1"/>
       <c r="J168" s="1"/>
       <c r="K168" s="1"/>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L168" s="1"/>
+      <c r="M168" s="1"/>
+    </row>
+    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
       <c r="C169" s="1"/>
@@ -2642,6 +2988,8 @@
       <c r="I169" s="1"/>
       <c r="J169" s="1"/>
       <c r="K169" s="1"/>
+      <c r="L169" s="1"/>
+      <c r="M169" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>